<commit_message>
Mirror the complete project layout and keep temporary files local
</commit_message>
<xml_diff>
--- a/基金/持仓基金/006485_广发中债1-3年国开行债券指数C/006485_交易记录.xlsx
+++ b/基金/持仓基金/006485_广发中债1-3年国开行债券指数C/006485_交易记录.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\AI 投研\基金\006485_广发中债1-3年国开行债券指数C\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\AI 投研\基金\持仓基金\006485_广发中债1-3年国开行债券指数C\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="15825" windowHeight="12165"/>
+    <workbookView windowWidth="16065" windowHeight="12750"/>
   </bookViews>
   <sheets>
     <sheet name="交易记录" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="8">
   <si>
     <t>交易日期</t>
   </si>
@@ -699,7 +699,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -720,6 +720,7 @@
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="31" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1000,7 +1001,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Transactions_006485" displayName="Transactions_006485" ref="A1:F19" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Transactions_006485" displayName="Transactions_006485" ref="A1:F20" totalsRowShown="0">
   <tableColumns count="6">
     <tableColumn id="1" name="交易日期"/>
     <tableColumn id="2" name="成交净值"/>
@@ -1210,7 +1211,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -1248,7 +1249,7 @@
         <v>1.0569</v>
       </c>
       <c r="C2" s="5">
-        <f>E2/B2</f>
+        <f t="shared" ref="C2:C18" si="0">E2/B2</f>
         <v>0.946163307786924</v>
       </c>
       <c r="D2" s="6" t="s">
@@ -1269,7 +1270,7 @@
         <v>1.0568</v>
       </c>
       <c r="C3" s="5">
-        <f>E3/B3</f>
+        <f t="shared" si="0"/>
         <v>946.252838758516</v>
       </c>
       <c r="D3" s="6" t="s">
@@ -1290,7 +1291,7 @@
         <v>1.0568</v>
       </c>
       <c r="C4" s="5">
-        <f>E4/B4</f>
+        <f t="shared" si="0"/>
         <v>473.126419379258</v>
       </c>
       <c r="D4" s="6" t="s">
@@ -1311,7 +1312,7 @@
         <v>1.0553</v>
       </c>
       <c r="C5" s="5">
-        <f>E5/B5</f>
+        <f t="shared" si="0"/>
         <v>947.597839476926</v>
       </c>
       <c r="D5" s="6" t="s">
@@ -1332,7 +1333,7 @@
         <v>1.0561</v>
       </c>
       <c r="C6" s="5">
-        <f>E6/B6</f>
+        <f t="shared" si="0"/>
         <v>894.025187008806</v>
       </c>
       <c r="D6" s="6" t="s">
@@ -1353,7 +1354,7 @@
         <v>1.0574</v>
       </c>
       <c r="C7" s="5">
-        <f>E7/B7</f>
+        <f t="shared" si="0"/>
         <v>998.997541138642</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -1374,7 +1375,7 @@
         <v>1.0583</v>
       </c>
       <c r="C8" s="5">
-        <f>E8/B8</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="D8" s="6" t="s">
@@ -1395,7 +1396,7 @@
         <v>1.0574</v>
       </c>
       <c r="C9" s="5">
-        <f>E9/B9</f>
+        <f t="shared" si="0"/>
         <v>945.715906941555</v>
       </c>
       <c r="D9" s="6" t="s">
@@ -1416,7 +1417,7 @@
         <v>1.0575</v>
       </c>
       <c r="C10" s="5">
-        <f>E10/B10</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="D10" s="6" t="s">
@@ -1437,7 +1438,7 @@
         <v>1.0575</v>
       </c>
       <c r="C11" s="5">
-        <f>E11/B11</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="D11" s="6" t="s">
@@ -1458,7 +1459,7 @@
         <v>1.0586</v>
       </c>
       <c r="C12" s="5">
-        <f>E12/B12</f>
+        <f t="shared" si="0"/>
         <v>1707.67995465709</v>
       </c>
       <c r="D12" s="6" t="s">
@@ -1479,7 +1480,7 @@
         <v>1.0559</v>
       </c>
       <c r="C13" s="5">
-        <f>E13/B13</f>
+        <f t="shared" si="0"/>
         <v>3788.23752249266</v>
       </c>
       <c r="D13" s="6" t="s">
@@ -1500,7 +1501,7 @@
         <v>1.056</v>
       </c>
       <c r="C14" s="5">
-        <f>E14/B14</f>
+        <f t="shared" si="0"/>
         <v>9430.97537878788</v>
       </c>
       <c r="D14" s="6" t="s">
@@ -1521,7 +1522,7 @@
         <v>1.0573</v>
       </c>
       <c r="C15" s="5">
-        <f>E15/B15</f>
+        <f t="shared" si="0"/>
         <v>9567.06705759955</v>
       </c>
       <c r="D15" s="6" t="s">
@@ -1542,7 +1543,7 @@
         <v>1.0587</v>
       </c>
       <c r="C16" s="5">
-        <f>E16/B16</f>
+        <f t="shared" si="0"/>
         <v>9286.84235383017</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -1563,7 +1564,7 @@
         <v>1.0587</v>
       </c>
       <c r="C17" s="5">
-        <f>E17/B17</f>
+        <f t="shared" si="0"/>
         <v>1889.10928497214</v>
       </c>
       <c r="D17" s="6" t="s">
@@ -1584,7 +1585,7 @@
         <v>1.0587</v>
       </c>
       <c r="C18" s="5">
-        <f>E18/B18</f>
+        <f t="shared" si="0"/>
         <v>755.643713988854</v>
       </c>
       <c r="D18" s="6" t="s">
@@ -1611,10 +1612,28 @@
         <v>0</v>
       </c>
     </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="8">
+        <v>46316</v>
+      </c>
+      <c r="C20" s="1" t="e">
+        <f>E20/B20</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20">
+        <v>30000</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="D19 D2:D18">
-      <formula1>"买入,卖出"</formula1>
+    <dataValidation type="list" sqref="D2:D20">
+      <formula1>"买入,卖出,转入"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>